<commit_message>
fix(scripts): group margin analysis by SKU with blank row separators
</commit_message>
<xml_diff>
--- a/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
+++ b/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
@@ -510,7 +510,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dibuat: 04/05/2026 14:37</t>
+          <t>Dibuat: 04/05/2026 14:40</t>
         </is>
       </c>
     </row>
@@ -24269,7 +24269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:Q93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -24463,328 +24463,80 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT0280</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Autan Lotion Nyamuk Renceng 6ml isi 12</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Sakura</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>4-5 pcs</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>7400</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>666</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>333</v>
-      </c>
-      <c r="L7" s="10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>313</v>
-      </c>
-      <c r="N7" s="5" t="n">
-        <v>6089</v>
-      </c>
-      <c r="O7" s="5" t="n">
-        <v>412</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <v>5677</v>
-      </c>
-      <c r="Q7" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 5,677</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT0286</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>All Night 50ml</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>13200</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>1188</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>594</v>
-      </c>
-      <c r="L8" s="10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N8" s="5" t="n">
-        <v>10168</v>
-      </c>
-      <c r="O8" s="5" t="n">
-        <v>9793</v>
-      </c>
-      <c r="P8" s="5" t="n">
-        <v>375</v>
-      </c>
-      <c r="Q8" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 375</t>
-        </is>
-      </c>
-    </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>BAAUT0280</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Autan Lotion Nyamuk Renceng 6ml isi 12</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>4-5 pcs</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT0286</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>All Night 50ml</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>2-3 pcs</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="H9" s="5" t="n">
-        <v>13200</v>
+        <v>7400</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>1188</v>
+        <v>666</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>594</v>
+        <v>333</v>
       </c>
       <c r="L9" s="10" t="n">
         <v>4.5</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>625</v>
+        <v>313</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>10793</v>
+        <v>6089</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>9793</v>
+        <v>412</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>1000</v>
+        <v>5677</v>
       </c>
       <c r="Q9" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT0420</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Sakura 50ml</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>13200</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>1188</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>594</v>
-      </c>
-      <c r="L10" s="10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N10" s="5" t="n">
-        <v>10168</v>
-      </c>
-      <c r="O10" s="5" t="n">
-        <v>9793</v>
-      </c>
-      <c r="P10" s="5" t="n">
-        <v>375</v>
-      </c>
-      <c r="Q10" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 375</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT2397</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Care Protect 50ml</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>13200</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>1188</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>594</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>10168</v>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>9793</v>
-      </c>
-      <c r="P11" s="5" t="n">
-        <v>375</v>
-      </c>
-      <c r="Q11" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 375</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 5,677</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>BAAUT2397</t>
+          <t>BAAUT0286</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -24794,19 +24546,19 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Care Protect 50ml</t>
+          <t>All Night 50ml</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>2-3 pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H12" s="5" t="n">
         <v>13200</v>
@@ -24824,30 +24576,30 @@
         <v>4.5</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>625</v>
+        <v>1250</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>10793</v>
+        <v>10168</v>
       </c>
       <c r="O12" s="5" t="n">
         <v>9793</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>1000</v>
+        <v>375</v>
       </c>
       <c r="Q12" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,000</t>
+          <t>DI ATAS TARGET +Rp 375</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>BAAUT2606</t>
+          <t>BAAUT0286</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -24857,19 +24609,19 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Floral Protect 50ml</t>
+          <t>All Night 50ml</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>1 pcs</t>
+          <t>2-3 pcs</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="5" t="n">
         <v>13200</v>
@@ -24887,343 +24639,107 @@
         <v>4.5</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>1250</v>
+        <v>625</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>10168</v>
+        <v>10793</v>
       </c>
       <c r="O13" s="5" t="n">
         <v>9793</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>375</v>
+        <v>1000</v>
       </c>
       <c r="Q13" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 375</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT4009</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>17100</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>1539</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>770</v>
-      </c>
-      <c r="L14" s="10" t="n">
-        <v>4.502923976608187</v>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>13541</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>13088</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>453</v>
-      </c>
-      <c r="Q14" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 453</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>BAAUT4009</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>2-3 pcs</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>17100</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>1539</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>770</v>
-      </c>
-      <c r="L15" s="10" t="n">
-        <v>4.502923976608187</v>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>625</v>
-      </c>
-      <c r="N15" s="5" t="n">
-        <v>14167</v>
-      </c>
-      <c r="O15" s="5" t="n">
-        <v>13088</v>
-      </c>
-      <c r="P15" s="5" t="n">
-        <v>1079</v>
-      </c>
-      <c r="Q15" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 1,079</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>BAAUT4009</t>
+          <t>BAAUT0420</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
+          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Sakura 50ml</t>
+        </is>
+      </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>6+ pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F16" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>17100</v>
+        <v>13200</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>1539</v>
+        <v>1188</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>770</v>
+        <v>594</v>
       </c>
       <c r="L16" s="10" t="n">
-        <v>4.502923976608187</v>
+        <v>4.5</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>208</v>
+        <v>1250</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>14583</v>
+        <v>10168</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>13088</v>
+        <v>9793</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>1495</v>
+        <v>375</v>
       </c>
       <c r="Q16" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,495</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5971</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>2439</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K17" s="5" t="n">
-        <v>1355</v>
-      </c>
-      <c r="L17" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N17" s="5" t="n">
-        <v>22056</v>
-      </c>
-      <c r="O17" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P17" s="5" t="n">
-        <v>556</v>
-      </c>
-      <c r="Q17" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 556</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5971</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>2-3 pcs</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>2372</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>8.752767527675278</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>1318</v>
-      </c>
-      <c r="L18" s="10" t="n">
-        <v>4.863468634686347</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>417</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>22244</v>
-      </c>
-      <c r="O18" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P18" s="5" t="n">
-        <v>744</v>
-      </c>
-      <c r="Q18" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 744</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 375</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>BAKIW5973</t>
+          <t>BAAUT2397</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
+          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Coklat</t>
+          <t>Care Protect 50ml</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -25232,61 +24748,61 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>12800</v>
+        <v>13200</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>1152</v>
+        <v>1188</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>640</v>
+        <v>594</v>
       </c>
       <c r="L19" s="10" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>1250</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>9758</v>
+        <v>10168</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>9460</v>
+        <v>9793</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>298</v>
+        <v>375</v>
       </c>
       <c r="Q19" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 298</t>
+          <t>DI ATAS TARGET +Rp 375</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>BAKIW5973</t>
+          <t>BAAUT2397</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
+          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Coklat</t>
+          <t>Care Protect 50ml</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -25295,681 +24811,297 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>12800</v>
+        <v>13200</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>1152</v>
+        <v>1188</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>640</v>
+        <v>594</v>
       </c>
       <c r="L20" s="10" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>486</v>
+        <v>625</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>10522</v>
+        <v>10793</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>9460</v>
+        <v>9793</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>1062</v>
+        <v>1000</v>
       </c>
       <c r="Q20" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,062</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5973</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Coklat</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>6+ pcs</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>12800</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>1152</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>640</v>
-      </c>
-      <c r="L21" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M21" s="5" t="n">
-        <v>52</v>
-      </c>
-      <c r="N21" s="5" t="n">
-        <v>10956</v>
-      </c>
-      <c r="O21" s="5" t="n">
-        <v>9460</v>
-      </c>
-      <c r="P21" s="5" t="n">
-        <v>1496</v>
-      </c>
-      <c r="Q21" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 1,496</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5975</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Hitam</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>142</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>142</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>2439</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <v>1355</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M22" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N22" s="5" t="n">
-        <v>22056</v>
-      </c>
-      <c r="O22" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P22" s="5" t="n">
-        <v>556</v>
-      </c>
-      <c r="Q22" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 556</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>BAKIW5975</t>
+          <t>BAAUT2606</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
+          <t>Autan Tube Lotion Anti Nyamuk 50ml</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Hitam</t>
+          <t>Floral Protect 50ml</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>2-3 pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>27100</v>
+        <v>13200</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>2372</v>
+        <v>1188</v>
       </c>
       <c r="J23" s="10" t="n">
-        <v>8.752767527675278</v>
+        <v>9</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>1318</v>
+        <v>594</v>
       </c>
       <c r="L23" s="10" t="n">
-        <v>4.863468634686347</v>
+        <v>4.5</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>577</v>
+        <v>1250</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>22084</v>
+        <v>10168</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>21500</v>
+        <v>9793</v>
       </c>
       <c r="P23" s="5" t="n">
-        <v>584</v>
+        <v>375</v>
       </c>
       <c r="Q23" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 584</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5975</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Hitam</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>4-5 pcs</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>2338</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>8.627306273062731</v>
-      </c>
-      <c r="K24" s="5" t="n">
-        <v>1299</v>
-      </c>
-      <c r="L24" s="10" t="n">
-        <v>4.793357933579336</v>
-      </c>
-      <c r="M24" s="5" t="n">
-        <v>297</v>
-      </c>
-      <c r="N24" s="5" t="n">
-        <v>22042</v>
-      </c>
-      <c r="O24" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P24" s="5" t="n">
-        <v>542</v>
-      </c>
-      <c r="Q24" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 542</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW5975</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Hitam</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>6+ pcs</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>538</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>2331</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>8.601476014760149</v>
-      </c>
-      <c r="K25" s="5" t="n">
-        <v>1295</v>
-      </c>
-      <c r="L25" s="10" t="n">
-        <v>4.778597785977859</v>
-      </c>
-      <c r="M25" s="5" t="n">
-        <v>101</v>
-      </c>
-      <c r="N25" s="5" t="n">
-        <v>22170</v>
-      </c>
-      <c r="O25" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P25" s="5" t="n">
-        <v>670</v>
-      </c>
-      <c r="Q25" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 670</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 375</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>BAKIW5976</t>
+          <t>BAAUT4009</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Coklat</t>
-        </is>
-      </c>
+          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>2-3 pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>40600</v>
+        <v>17100</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>3654</v>
+        <v>1539</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>2030</v>
+        <v>770</v>
       </c>
       <c r="L26" s="10" t="n">
-        <v>5</v>
+        <v>4.502923976608187</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>625</v>
+        <v>1250</v>
       </c>
       <c r="N26" s="5" t="n">
-        <v>34291</v>
+        <v>13541</v>
       </c>
       <c r="O26" s="5" t="n">
-        <v>32766</v>
+        <v>13088</v>
       </c>
       <c r="P26" s="5" t="n">
-        <v>1525</v>
+        <v>453</v>
       </c>
       <c r="Q26" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,525</t>
+          <t>DI ATAS TARGET +Rp 453</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>BAKIW5976</t>
+          <t>BAAUT4009</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Coklat</t>
-        </is>
-      </c>
+          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>6+ pcs</t>
+          <t>2-3 pcs</t>
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>40600</v>
+        <v>17100</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>3654</v>
+        <v>1539</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>2030</v>
+        <v>770</v>
       </c>
       <c r="L27" s="10" t="n">
-        <v>5</v>
+        <v>4.502923976608187</v>
       </c>
       <c r="M27" s="5" t="n">
-        <v>179</v>
+        <v>625</v>
       </c>
       <c r="N27" s="5" t="n">
-        <v>34737</v>
+        <v>14167</v>
       </c>
       <c r="O27" s="5" t="n">
-        <v>32766</v>
+        <v>13088</v>
       </c>
       <c r="P27" s="5" t="n">
-        <v>1971</v>
+        <v>1079</v>
       </c>
       <c r="Q27" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 1,971</t>
+          <t>DI ATAS TARGET +Rp 1,079</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>BAKIW6133</t>
+          <t>BAAUT4009</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
+          <t>Autan Spray Cair Anti Nyamuk Botol 100ml</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>1 pcs</t>
+          <t>6+ pcs</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>6</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>21000</v>
+        <v>17100</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>1890</v>
+        <v>1539</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1050</v>
+        <v>770</v>
       </c>
       <c r="L28" s="10" t="n">
-        <v>5</v>
+        <v>4.502923976608187</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>1250</v>
+        <v>208</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>16810</v>
+        <v>14583</v>
       </c>
       <c r="O28" s="5" t="n">
-        <v>16340</v>
+        <v>13088</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>470</v>
+        <v>1495</v>
       </c>
       <c r="Q28" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 470</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW6133</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>6+ pcs</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>21000</v>
-      </c>
-      <c r="I29" s="5" t="n">
-        <v>1890</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K29" s="5" t="n">
-        <v>1050</v>
-      </c>
-      <c r="L29" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M29" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="N29" s="5" t="n">
-        <v>17998</v>
-      </c>
-      <c r="O29" s="5" t="n">
-        <v>16340</v>
-      </c>
-      <c r="P29" s="5" t="n">
-        <v>1658</v>
-      </c>
-      <c r="Q29" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 1,658</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW6134</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Coklat</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>27100</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>2439</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>1355</v>
-      </c>
-      <c r="L30" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M30" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>22056</v>
-      </c>
-      <c r="O30" s="5" t="n">
-        <v>21500</v>
-      </c>
-      <c r="P30" s="5" t="n">
-        <v>556</v>
-      </c>
-      <c r="Q30" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 556</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 1,495</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>BAKIW6134</t>
+          <t>BAKIW5971</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -25979,259 +25111,135 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Coklat</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>2-3 pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H31" s="5" t="n">
         <v>27100</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>2372</v>
+        <v>2439</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>8.752767527675278</v>
+        <v>9</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>1318</v>
+        <v>1355</v>
       </c>
       <c r="L31" s="10" t="n">
-        <v>4.863468634686347</v>
+        <v>5</v>
       </c>
       <c r="M31" s="5" t="n">
-        <v>625</v>
+        <v>1250</v>
       </c>
       <c r="N31" s="5" t="n">
-        <v>22036</v>
+        <v>22056</v>
       </c>
       <c r="O31" s="5" t="n">
         <v>21500</v>
       </c>
       <c r="P31" s="5" t="n">
-        <v>536</v>
+        <v>556</v>
       </c>
       <c r="Q31" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 536</t>
+          <t>DI ATAS TARGET +Rp 556</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>BAKIW6135</t>
+          <t>BAKIW5971</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Hitam</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>1 pcs</t>
+          <t>2-3 pcs</t>
         </is>
       </c>
       <c r="F32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>21000</v>
+        <v>27100</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>1890</v>
+        <v>2372</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>9</v>
+        <v>8.752767527675278</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1050</v>
+        <v>1318</v>
       </c>
       <c r="L32" s="10" t="n">
-        <v>5</v>
+        <v>4.863468634686347</v>
       </c>
       <c r="M32" s="5" t="n">
-        <v>1250</v>
+        <v>417</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>16810</v>
+        <v>22244</v>
       </c>
       <c r="O32" s="5" t="n">
-        <v>16340</v>
+        <v>21500</v>
       </c>
       <c r="P32" s="5" t="n">
-        <v>470</v>
+        <v>744</v>
       </c>
       <c r="Q32" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 470</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW6288</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Hitam</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>40600</v>
-      </c>
-      <c r="I33" s="5" t="n">
-        <v>3654</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K33" s="5" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L33" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M33" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N33" s="5" t="n">
-        <v>33666</v>
-      </c>
-      <c r="O33" s="5" t="n">
-        <v>32766</v>
-      </c>
-      <c r="P33" s="5" t="n">
-        <v>900</v>
-      </c>
-      <c r="Q33" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 900</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>BAKIW6288</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Hitam</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>2-3 pcs</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>40600</v>
-      </c>
-      <c r="I34" s="5" t="n">
-        <v>3654</v>
-      </c>
-      <c r="J34" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K34" s="5" t="n">
-        <v>2030</v>
-      </c>
-      <c r="L34" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="M34" s="5" t="n">
-        <v>625</v>
-      </c>
-      <c r="N34" s="5" t="n">
-        <v>34291</v>
-      </c>
-      <c r="O34" s="5" t="n">
-        <v>32766</v>
-      </c>
-      <c r="P34" s="5" t="n">
-        <v>1525</v>
-      </c>
-      <c r="Q34" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 1,525</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 744</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5558</t>
+          <t>BAKIW5973</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Coklat 240gr</t>
+          <t>Coklat</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -26240,61 +25248,61 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>11000</v>
+        <v>12800</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>908</v>
+        <v>1152</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>8.254545454545454</v>
+        <v>9</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>495</v>
+        <v>640</v>
       </c>
       <c r="L35" s="10" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="M35" s="5" t="n">
         <v>1250</v>
       </c>
       <c r="N35" s="5" t="n">
-        <v>8347</v>
+        <v>9758</v>
       </c>
       <c r="O35" s="5" t="n">
-        <v>7797</v>
+        <v>9460</v>
       </c>
       <c r="P35" s="5" t="n">
-        <v>550</v>
+        <v>298</v>
       </c>
       <c r="Q35" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 550</t>
+          <t>DI ATAS TARGET +Rp 298</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5558</t>
+          <t>BAKIW5973</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Coklat 240gr</t>
+          <t>Coklat</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -26303,628 +25311,380 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>11000</v>
+        <v>12800</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>829</v>
+        <v>1152</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>7.536363636363637</v>
+        <v>9</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>452</v>
+        <v>640</v>
       </c>
       <c r="L36" s="10" t="n">
-        <v>4.109090909090908</v>
+        <v>5</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>609</v>
+        <v>486</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>8160</v>
+        <v>10522</v>
       </c>
       <c r="O36" s="5" t="n">
-        <v>7797</v>
+        <v>9460</v>
       </c>
       <c r="P36" s="5" t="n">
-        <v>363</v>
+        <v>1062</v>
       </c>
       <c r="Q36" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 363</t>
+          <t>DI ATAS TARGET +Rp 1,062</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5558</t>
+          <t>BAKIW5973</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 17.5ml</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Coklat 240gr</t>
+          <t>Coklat</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>4-5 pcs</t>
+          <t>6+ pcs</t>
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>11000</v>
+        <v>12800</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>798</v>
+        <v>1152</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>7.254545454545455</v>
+        <v>9</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>436</v>
+        <v>640</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>3.963636363636364</v>
+        <v>5</v>
       </c>
       <c r="M37" s="5" t="n">
-        <v>313</v>
+        <v>52</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>8129</v>
+        <v>10956</v>
       </c>
       <c r="O37" s="5" t="n">
-        <v>7797</v>
+        <v>9460</v>
       </c>
       <c r="P37" s="5" t="n">
-        <v>332</v>
+        <v>1496</v>
       </c>
       <c r="Q37" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 332</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>FFBSK5558</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Coklat 240gr</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>6+ pcs</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="I38" s="5" t="n">
-        <v>788</v>
-      </c>
-      <c r="J38" s="10" t="n">
-        <v>7.163636363636364</v>
-      </c>
-      <c r="K38" s="5" t="n">
-        <v>430</v>
-      </c>
-      <c r="L38" s="10" t="n">
-        <v>3.909090909090909</v>
-      </c>
-      <c r="M38" s="5" t="n">
-        <v>179</v>
-      </c>
-      <c r="N38" s="5" t="n">
-        <v>8154</v>
-      </c>
-      <c r="O38" s="5" t="n">
-        <v>7797</v>
-      </c>
-      <c r="P38" s="5" t="n">
-        <v>357</v>
-      </c>
-      <c r="Q38" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 357</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>FFBSK5993</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Putih 240gr</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="H39" s="5" t="n">
-        <v>11000</v>
-      </c>
-      <c r="I39" s="5" t="n">
-        <v>908</v>
-      </c>
-      <c r="J39" s="10" t="n">
-        <v>8.254545454545454</v>
-      </c>
-      <c r="K39" s="5" t="n">
-        <v>495</v>
-      </c>
-      <c r="L39" s="10" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M39" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N39" s="5" t="n">
-        <v>8347</v>
-      </c>
-      <c r="O39" s="5" t="n">
-        <v>7797</v>
-      </c>
-      <c r="P39" s="5" t="n">
-        <v>550</v>
-      </c>
-      <c r="Q39" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 550</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 1,496</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5993</t>
+          <t>BAKIW5975</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Putih 240gr</t>
+          <t>Hitam</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>2-3 pcs</t>
+          <t>1 pcs</t>
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>24</v>
+        <v>142</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>54</v>
+        <v>142</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>11000</v>
+        <v>27100</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>829</v>
+        <v>2439</v>
       </c>
       <c r="J40" s="10" t="n">
-        <v>7.536363636363637</v>
+        <v>9</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>452</v>
+        <v>1355</v>
       </c>
       <c r="L40" s="10" t="n">
-        <v>4.109090909090908</v>
+        <v>5</v>
       </c>
       <c r="M40" s="5" t="n">
-        <v>573</v>
+        <v>1250</v>
       </c>
       <c r="N40" s="5" t="n">
-        <v>8196</v>
+        <v>22056</v>
       </c>
       <c r="O40" s="5" t="n">
-        <v>7797</v>
+        <v>21500</v>
       </c>
       <c r="P40" s="5" t="n">
-        <v>399</v>
+        <v>556</v>
       </c>
       <c r="Q40" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 399</t>
+          <t>DI ATAS TARGET +Rp 556</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5993</t>
+          <t>BAKIW5975</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Putih 240gr</t>
+          <t>Hitam</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>4-5 pcs</t>
+          <t>2-3 pcs</t>
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>11000</v>
+        <v>27100</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>798</v>
+        <v>2372</v>
       </c>
       <c r="J41" s="10" t="n">
-        <v>7.254545454545455</v>
+        <v>8.752767527675278</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>435</v>
+        <v>1318</v>
       </c>
       <c r="L41" s="10" t="n">
-        <v>3.954545454545454</v>
+        <v>4.863468634686347</v>
       </c>
       <c r="M41" s="5" t="n">
-        <v>275</v>
+        <v>577</v>
       </c>
       <c r="N41" s="5" t="n">
-        <v>8166</v>
+        <v>22084</v>
       </c>
       <c r="O41" s="5" t="n">
-        <v>7797</v>
+        <v>21500</v>
       </c>
       <c r="P41" s="5" t="n">
-        <v>369</v>
+        <v>584</v>
       </c>
       <c r="Q41" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 369</t>
+          <t>DI ATAS TARGET +Rp 584</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>FFBSK5993</t>
+          <t>BAKIW5975</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Putih 240gr</t>
+          <t>Hitam</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>6+ pcs</t>
+          <t>4-5 pcs</t>
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>11000</v>
+        <v>27100</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>788</v>
+        <v>2338</v>
       </c>
       <c r="J42" s="10" t="n">
-        <v>7.163636363636364</v>
+        <v>8.627306273062731</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>430</v>
+        <v>1299</v>
       </c>
       <c r="L42" s="10" t="n">
-        <v>3.909090909090909</v>
+        <v>4.793357933579336</v>
       </c>
       <c r="M42" s="5" t="n">
-        <v>119</v>
+        <v>297</v>
       </c>
       <c r="N42" s="5" t="n">
-        <v>8214</v>
+        <v>22042</v>
       </c>
       <c r="O42" s="5" t="n">
-        <v>7797</v>
+        <v>21500</v>
       </c>
       <c r="P42" s="5" t="n">
-        <v>417</v>
+        <v>542</v>
       </c>
       <c r="Q42" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 417</t>
+          <t>DI ATAS TARGET +Rp 542</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>FG102370280602C</t>
+          <t>BAKIW5975</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>B&amp;B Kids Body Powder Bedak Anak</t>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Bubbles 60 gr</t>
+          <t>Hitam</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>1 pcs</t>
+          <t>6+ pcs</t>
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>1</v>
+        <v>538</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>8000</v>
+        <v>27100</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>660</v>
+        <v>2331</v>
       </c>
       <c r="J43" s="10" t="n">
-        <v>8.25</v>
+        <v>8.601476014760149</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>320</v>
+        <v>1295</v>
       </c>
       <c r="L43" s="10" t="n">
-        <v>4</v>
+        <v>4.778597785977859</v>
       </c>
       <c r="M43" s="5" t="n">
-        <v>1250</v>
+        <v>101</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>5770</v>
+        <v>22170</v>
       </c>
       <c r="O43" s="5" t="n">
-        <v>5325</v>
+        <v>21500</v>
       </c>
       <c r="P43" s="5" t="n">
-        <v>445</v>
+        <v>670</v>
       </c>
       <c r="Q43" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 445</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>UN1088147</t>
-        </is>
-      </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>Charm Pembalut Wanita Cooling Fresh Sensasi Dingin 23 cm</t>
-        </is>
-      </c>
-      <c r="D44" s="12" t="inlineStr">
-        <is>
-          <t>Wing 16 Pads</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="13" t="n">
-        <v>13000</v>
-      </c>
-      <c r="I44" s="13" t="n">
-        <v>1170</v>
-      </c>
-      <c r="J44" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="K44" s="13" t="n">
-        <v>585</v>
-      </c>
-      <c r="L44" s="14" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="M44" s="13" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N44" s="13" t="n">
-        <v>9995</v>
-      </c>
-      <c r="O44" s="13" t="n">
-        <v>11610</v>
-      </c>
-      <c r="P44" s="13" t="n">
-        <v>-1615</v>
-      </c>
-      <c r="Q44" s="12" t="inlineStr">
-        <is>
-          <t>DI BAWAH TARGET (RUGI Rp 1,615)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>UN2814232</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>MamyPoko Pants Xtra Kering Celana Popok Bayi Renceng isi 10 S/M/L/XL</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>1 pcs</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G45" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H45" s="5" t="n">
-        <v>14800</v>
-      </c>
-      <c r="I45" s="5" t="n">
-        <v>1332</v>
-      </c>
-      <c r="J45" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="K45" s="5" t="n">
-        <v>592</v>
-      </c>
-      <c r="L45" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="M45" s="5" t="n">
-        <v>1250</v>
-      </c>
-      <c r="N45" s="5" t="n">
-        <v>11626</v>
-      </c>
-      <c r="O45" s="5" t="n">
-        <v>924</v>
-      </c>
-      <c r="P45" s="5" t="n">
-        <v>10702</v>
-      </c>
-      <c r="Q45" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 10,702</t>
-        </is>
-      </c>
-    </row>
+          <t>DI ATAS TARGET +Rp 670</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>UN2814232</t>
+          <t>BAKIW5976</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>MamyPoko Pants Xtra Kering Celana Popok Bayi Renceng isi 10 S/M/L/XL</t>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Coklat</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -26939,222 +25699,1506 @@
         <v>2</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>14800</v>
+        <v>40600</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>1332</v>
+        <v>3654</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>9</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>592</v>
+        <v>2030</v>
       </c>
       <c r="L46" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M46" s="5" t="n">
         <v>625</v>
       </c>
       <c r="N46" s="5" t="n">
-        <v>12251</v>
+        <v>34291</v>
       </c>
       <c r="O46" s="5" t="n">
-        <v>924</v>
+        <v>32766</v>
       </c>
       <c r="P46" s="5" t="n">
-        <v>11327</v>
+        <v>1525</v>
       </c>
       <c r="Q46" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 11,327</t>
+          <t>DI ATAS TARGET +Rp 1,525</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW5976</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Coklat</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>6+ pcs</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>40600</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>3654</v>
+      </c>
+      <c r="J47" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K47" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L47" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M47" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="N47" s="5" t="n">
+        <v>34737</v>
+      </c>
+      <c r="O47" s="5" t="n">
+        <v>32766</v>
+      </c>
+      <c r="P47" s="5" t="n">
+        <v>1971</v>
+      </c>
+      <c r="Q47" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 1,971</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6133</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>21000</v>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>1890</v>
+      </c>
+      <c r="J50" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K50" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="L50" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M50" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N50" s="5" t="n">
+        <v>16810</v>
+      </c>
+      <c r="O50" s="5" t="n">
+        <v>16340</v>
+      </c>
+      <c r="P50" s="5" t="n">
+        <v>470</v>
+      </c>
+      <c r="Q50" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 470</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6133</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>6+ pcs</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>21000</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>1890</v>
+      </c>
+      <c r="J51" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K51" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="L51" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="N51" s="5" t="n">
+        <v>17998</v>
+      </c>
+      <c r="O51" s="5" t="n">
+        <v>16340</v>
+      </c>
+      <c r="P51" s="5" t="n">
+        <v>1658</v>
+      </c>
+      <c r="Q51" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 1,658</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6134</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Coklat</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>27100</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>2439</v>
+      </c>
+      <c r="J54" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K54" s="5" t="n">
+        <v>1355</v>
+      </c>
+      <c r="L54" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M54" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N54" s="5" t="n">
+        <v>22056</v>
+      </c>
+      <c r="O54" s="5" t="n">
+        <v>21500</v>
+      </c>
+      <c r="P54" s="5" t="n">
+        <v>556</v>
+      </c>
+      <c r="Q54" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 556</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6134</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Paste SP 45ml - Perawatan Sepatu</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Coklat</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>2-3 pcs</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>27100</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>2372</v>
+      </c>
+      <c r="J55" s="10" t="n">
+        <v>8.752767527675278</v>
+      </c>
+      <c r="K55" s="5" t="n">
+        <v>1318</v>
+      </c>
+      <c r="L55" s="10" t="n">
+        <v>4.863468634686347</v>
+      </c>
+      <c r="M55" s="5" t="n">
+        <v>625</v>
+      </c>
+      <c r="N55" s="5" t="n">
+        <v>22036</v>
+      </c>
+      <c r="O55" s="5" t="n">
+        <v>21500</v>
+      </c>
+      <c r="P55" s="5" t="n">
+        <v>536</v>
+      </c>
+      <c r="Q55" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 536</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6135</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 30ml</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Hitam</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="5" t="n">
+        <v>21000</v>
+      </c>
+      <c r="I58" s="5" t="n">
+        <v>1890</v>
+      </c>
+      <c r="J58" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K58" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="L58" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M58" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N58" s="5" t="n">
+        <v>16810</v>
+      </c>
+      <c r="O58" s="5" t="n">
+        <v>16340</v>
+      </c>
+      <c r="P58" s="5" t="n">
+        <v>470</v>
+      </c>
+      <c r="Q58" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 470</t>
+        </is>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6288</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Hitam</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>40600</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>3654</v>
+      </c>
+      <c r="J61" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K61" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L61" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M61" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N61" s="5" t="n">
+        <v>33666</v>
+      </c>
+      <c r="O61" s="5" t="n">
+        <v>32766</v>
+      </c>
+      <c r="P61" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="Q61" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 900</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>BAKIW6288</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>KIWI Semir Sepatu Liquid Shine &amp; Protect 75ml</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Hitam</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>2-3 pcs</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H62" s="5" t="n">
+        <v>40600</v>
+      </c>
+      <c r="I62" s="5" t="n">
+        <v>3654</v>
+      </c>
+      <c r="J62" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K62" s="5" t="n">
+        <v>2030</v>
+      </c>
+      <c r="L62" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M62" s="5" t="n">
+        <v>625</v>
+      </c>
+      <c r="N62" s="5" t="n">
+        <v>34291</v>
+      </c>
+      <c r="O62" s="5" t="n">
+        <v>32766</v>
+      </c>
+      <c r="P62" s="5" t="n">
+        <v>1525</v>
+      </c>
+      <c r="Q62" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 1,525</t>
+        </is>
+      </c>
+    </row>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5558</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Coklat 240gr</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>908</v>
+      </c>
+      <c r="J65" s="10" t="n">
+        <v>8.254545454545454</v>
+      </c>
+      <c r="K65" s="5" t="n">
+        <v>495</v>
+      </c>
+      <c r="L65" s="10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M65" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N65" s="5" t="n">
+        <v>8347</v>
+      </c>
+      <c r="O65" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P65" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="Q65" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 550</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5558</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Coklat 240gr</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>2-3 pcs</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="H66" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="J66" s="10" t="n">
+        <v>7.536363636363637</v>
+      </c>
+      <c r="K66" s="5" t="n">
+        <v>452</v>
+      </c>
+      <c r="L66" s="10" t="n">
+        <v>4.109090909090908</v>
+      </c>
+      <c r="M66" s="5" t="n">
+        <v>609</v>
+      </c>
+      <c r="N66" s="5" t="n">
+        <v>8160</v>
+      </c>
+      <c r="O66" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P66" s="5" t="n">
+        <v>363</v>
+      </c>
+      <c r="Q66" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 363</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5558</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Coklat 240gr</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>4-5 pcs</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="J67" s="10" t="n">
+        <v>7.254545454545455</v>
+      </c>
+      <c r="K67" s="5" t="n">
+        <v>436</v>
+      </c>
+      <c r="L67" s="10" t="n">
+        <v>3.963636363636364</v>
+      </c>
+      <c r="M67" s="5" t="n">
+        <v>313</v>
+      </c>
+      <c r="N67" s="5" t="n">
+        <v>8129</v>
+      </c>
+      <c r="O67" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P67" s="5" t="n">
+        <v>332</v>
+      </c>
+      <c r="Q67" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 332</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5558</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Coklat 240gr</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>6+ pcs</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I68" s="5" t="n">
+        <v>788</v>
+      </c>
+      <c r="J68" s="10" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="K68" s="5" t="n">
+        <v>430</v>
+      </c>
+      <c r="L68" s="10" t="n">
+        <v>3.909090909090909</v>
+      </c>
+      <c r="M68" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="N68" s="5" t="n">
+        <v>8154</v>
+      </c>
+      <c r="O68" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P68" s="5" t="n">
+        <v>357</v>
+      </c>
+      <c r="Q68" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 357</t>
+        </is>
+      </c>
+    </row>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5993</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Putih 240gr</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="H71" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>908</v>
+      </c>
+      <c r="J71" s="10" t="n">
+        <v>8.254545454545454</v>
+      </c>
+      <c r="K71" s="5" t="n">
+        <v>495</v>
+      </c>
+      <c r="L71" s="10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M71" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N71" s="5" t="n">
+        <v>8347</v>
+      </c>
+      <c r="O71" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P71" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="Q71" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 550</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5993</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Putih 240gr</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>2-3 pcs</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="H72" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I72" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="J72" s="10" t="n">
+        <v>7.536363636363637</v>
+      </c>
+      <c r="K72" s="5" t="n">
+        <v>452</v>
+      </c>
+      <c r="L72" s="10" t="n">
+        <v>4.109090909090908</v>
+      </c>
+      <c r="M72" s="5" t="n">
+        <v>573</v>
+      </c>
+      <c r="N72" s="5" t="n">
+        <v>8196</v>
+      </c>
+      <c r="O72" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P72" s="5" t="n">
+        <v>399</v>
+      </c>
+      <c r="Q72" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 399</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5993</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Putih 240gr</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>4-5 pcs</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H73" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>798</v>
+      </c>
+      <c r="J73" s="10" t="n">
+        <v>7.254545454545455</v>
+      </c>
+      <c r="K73" s="5" t="n">
+        <v>435</v>
+      </c>
+      <c r="L73" s="10" t="n">
+        <v>3.954545454545454</v>
+      </c>
+      <c r="M73" s="5" t="n">
+        <v>275</v>
+      </c>
+      <c r="N73" s="5" t="n">
+        <v>8166</v>
+      </c>
+      <c r="O73" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P73" s="5" t="n">
+        <v>369</v>
+      </c>
+      <c r="Q73" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 369</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>FFBSK5993</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Frisian Flag Bendera Kental Manis Pouch 240gr</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Putih 240gr</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>6+ pcs</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="H74" s="5" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I74" s="5" t="n">
+        <v>788</v>
+      </c>
+      <c r="J74" s="10" t="n">
+        <v>7.163636363636364</v>
+      </c>
+      <c r="K74" s="5" t="n">
+        <v>430</v>
+      </c>
+      <c r="L74" s="10" t="n">
+        <v>3.909090909090909</v>
+      </c>
+      <c r="M74" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="N74" s="5" t="n">
+        <v>8214</v>
+      </c>
+      <c r="O74" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="P74" s="5" t="n">
+        <v>417</v>
+      </c>
+      <c r="Q74" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 417</t>
+        </is>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>FG102370280602C</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>B&amp;B Kids Body Powder Bedak Anak</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Bubbles 60 gr</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>660</v>
+      </c>
+      <c r="J77" s="10" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="K77" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="L77" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="M77" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N77" s="5" t="n">
+        <v>5770</v>
+      </c>
+      <c r="O77" s="5" t="n">
+        <v>5325</v>
+      </c>
+      <c r="P77" s="5" t="n">
+        <v>445</v>
+      </c>
+      <c r="Q77" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 445</t>
+        </is>
+      </c>
+    </row>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80">
+      <c r="A80" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>UN1088147</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>Charm Pembalut Wanita Cooling Fresh Sensasi Dingin 23 cm</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>Wing 16 Pads</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" s="13" t="n">
+        <v>13000</v>
+      </c>
+      <c r="I80" s="13" t="n">
+        <v>1170</v>
+      </c>
+      <c r="J80" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="K80" s="13" t="n">
+        <v>585</v>
+      </c>
+      <c r="L80" s="14" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="M80" s="13" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N80" s="13" t="n">
+        <v>9995</v>
+      </c>
+      <c r="O80" s="13" t="n">
+        <v>11610</v>
+      </c>
+      <c r="P80" s="13" t="n">
+        <v>-1615</v>
+      </c>
+      <c r="Q80" s="12" t="inlineStr">
+        <is>
+          <t>DI BAWAH TARGET (RUGI Rp 1,615)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>UN2814232</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>MamyPoko Pants Xtra Kering Celana Popok Bayi Renceng isi 10 S/M/L/XL</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>1 pcs</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H83" s="5" t="n">
+        <v>14800</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>1332</v>
+      </c>
+      <c r="J83" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K83" s="5" t="n">
+        <v>592</v>
+      </c>
+      <c r="L83" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="M83" s="5" t="n">
+        <v>1250</v>
+      </c>
+      <c r="N83" s="5" t="n">
+        <v>11626</v>
+      </c>
+      <c r="O83" s="5" t="n">
+        <v>924</v>
+      </c>
+      <c r="P83" s="5" t="n">
+        <v>10702</v>
+      </c>
+      <c r="Q83" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 10,702</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>UN2814232</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>MamyPoko Pants Xtra Kering Celana Popok Bayi Renceng isi 10 S/M/L/XL</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>2-3 pcs</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H84" s="5" t="n">
+        <v>14800</v>
+      </c>
+      <c r="I84" s="5" t="n">
+        <v>1332</v>
+      </c>
+      <c r="J84" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K84" s="5" t="n">
+        <v>592</v>
+      </c>
+      <c r="L84" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="M84" s="5" t="n">
+        <v>625</v>
+      </c>
+      <c r="N84" s="5" t="n">
+        <v>12251</v>
+      </c>
+      <c r="O84" s="5" t="n">
+        <v>924</v>
+      </c>
+      <c r="P84" s="5" t="n">
+        <v>11327</v>
+      </c>
+      <c r="Q84" s="11" t="inlineStr">
+        <is>
+          <t>DI ATAS TARGET +Rp 11,327</t>
+        </is>
+      </c>
+    </row>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87">
+      <c r="A87" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>UNMOL2709</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Molto Renceng 1000 Pelembut dan Pewangi Pakaian isi 6</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>6+ pcs</t>
         </is>
       </c>
-      <c r="F47" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="4" t="n">
+      <c r="F87" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H47" s="5" t="n">
+      <c r="H87" s="5" t="n">
         <v>6700</v>
       </c>
-      <c r="I47" s="5" t="n">
+      <c r="I87" s="5" t="n">
         <v>491</v>
       </c>
-      <c r="J47" s="10" t="n">
+      <c r="J87" s="10" t="n">
         <v>7.328358208955224</v>
       </c>
-      <c r="K47" s="5" t="n">
+      <c r="K87" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="L47" s="10" t="n">
+      <c r="L87" s="10" t="n">
         <v>4.477611940298507</v>
       </c>
-      <c r="M47" s="5" t="n">
+      <c r="M87" s="5" t="n">
         <v>208</v>
       </c>
-      <c r="N47" s="5" t="n">
+      <c r="N87" s="5" t="n">
         <v>4451</v>
       </c>
-      <c r="O47" s="5" t="n">
+      <c r="O87" s="5" t="n">
         <v>743</v>
       </c>
-      <c r="P47" s="5" t="n">
+      <c r="P87" s="5" t="n">
         <v>3708</v>
       </c>
-      <c r="Q47" s="11" t="inlineStr">
+      <c r="Q87" s="11" t="inlineStr">
         <is>
           <t>DI ATAS TARGET +Rp 3,708</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90">
+      <c r="A90" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>UNMOL2713</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>Molto Renceng 1000 Pelembut dan Pewangi Pakaian isi 6</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D90" s="4" t="inlineStr">
         <is>
           <t>Pink</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>6+ pcs</t>
         </is>
       </c>
-      <c r="F48" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="4" t="n">
+      <c r="F90" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H48" s="5" t="n">
+      <c r="H90" s="5" t="n">
         <v>6700</v>
       </c>
-      <c r="I48" s="5" t="n">
+      <c r="I90" s="5" t="n">
         <v>491</v>
       </c>
-      <c r="J48" s="10" t="n">
+      <c r="J90" s="10" t="n">
         <v>7.328358208955224</v>
       </c>
-      <c r="K48" s="5" t="n">
+      <c r="K90" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="L48" s="10" t="n">
+      <c r="L90" s="10" t="n">
         <v>4.477611940298507</v>
       </c>
-      <c r="M48" s="5" t="n">
+      <c r="M90" s="5" t="n">
         <v>208</v>
       </c>
-      <c r="N48" s="5" t="n">
+      <c r="N90" s="5" t="n">
         <v>4451</v>
       </c>
-      <c r="O48" s="5" t="n">
+      <c r="O90" s="5" t="n">
         <v>743</v>
       </c>
-      <c r="P48" s="5" t="n">
+      <c r="P90" s="5" t="n">
         <v>3708</v>
       </c>
-      <c r="Q48" s="11" t="inlineStr">
+      <c r="Q90" s="11" t="inlineStr">
         <is>
           <t>DI ATAS TARGET +Rp 3,708</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93">
+      <c r="A93" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>UNRIN4112</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Rinso Molto 500 Anti Noda Cair Isi 12 Sachet 18 ML</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D93" s="4" t="inlineStr">
         <is>
           <t>Royal Gold 12pcs</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E93" s="4" t="inlineStr">
         <is>
           <t>2-3 pcs</t>
         </is>
       </c>
-      <c r="F49" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="4" t="n">
+      <c r="F93" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H49" s="5" t="n">
+      <c r="H93" s="5" t="n">
         <v>5850</v>
       </c>
-      <c r="I49" s="5" t="n">
+      <c r="I93" s="5" t="n">
         <v>527</v>
       </c>
-      <c r="J49" s="10" t="n">
+      <c r="J93" s="10" t="n">
         <v>9.008547008547009</v>
       </c>
-      <c r="K49" s="5" t="n">
+      <c r="K93" s="5" t="n">
         <v>322</v>
       </c>
-      <c r="L49" s="10" t="n">
+      <c r="L93" s="10" t="n">
         <v>5.504273504273504</v>
       </c>
-      <c r="M49" s="5" t="n">
+      <c r="M93" s="5" t="n">
         <v>625</v>
       </c>
-      <c r="N49" s="5" t="n">
+      <c r="N93" s="5" t="n">
         <v>4377</v>
       </c>
-      <c r="O49" s="5" t="n">
+      <c r="O93" s="5" t="n">
         <v>362</v>
       </c>
-      <c r="P49" s="5" t="n">
+      <c r="P93" s="5" t="n">
         <v>4015</v>
       </c>
-      <c r="Q49" s="11" t="inlineStr">
+      <c r="Q93" s="11" t="inlineStr">
         <is>
           <t>DI ATAS TARGET +Rp 4,015</t>
         </is>

</xml_diff>

<commit_message>
fix(scripts): use discounted_price as subtotal, modal from kartonan (beli+3%), show full pricing formula
</commit_message>
<xml_diff>
--- a/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
+++ b/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
@@ -510,7 +510,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dibuat: 04/05/2026 14:40</t>
+          <t>Dibuat: 04/05/2026 15:01</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="5" t="n">
-        <v>34178600</v>
+        <v>32854750</v>
       </c>
     </row>
     <row r="10">
@@ -797,7 +797,7 @@
         <v>24</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>650400</v>
+        <v>620400</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>55836</v>
@@ -845,7 +845,7 @@
         <v>4</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>9351</v>
@@ -989,7 +989,7 @@
         <v>8</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>216800</v>
+        <v>206800</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>18612</v>
@@ -1037,7 +1037,7 @@
         <v>4</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>9351</v>
@@ -1085,7 +1085,7 @@
         <v>4</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>9351</v>
@@ -1133,7 +1133,7 @@
         <v>2</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>4743</v>
@@ -1277,7 +1277,7 @@
         <v>80</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2168000</v>
+        <v>2068000</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>186120</v>
@@ -1325,7 +1325,7 @@
         <v>2</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>4743</v>
@@ -1421,7 +1421,7 @@
         <v>5</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>135500</v>
+        <v>129875</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>11689</v>
@@ -1469,7 +1469,7 @@
         <v>20</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>542000</v>
+        <v>517000</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>46530</v>
@@ -1613,7 +1613,7 @@
         <v>2</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>4743</v>
@@ -1805,7 +1805,7 @@
         <v>12</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>325200</v>
+        <v>310200</v>
       </c>
       <c r="I24" s="5" t="n">
         <v>27918</v>
@@ -1901,7 +1901,7 @@
         <v>8</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>188200</v>
+        <v>180700</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>16263</v>
@@ -1997,7 +1997,7 @@
         <v>2</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I28" s="5" t="n">
         <v>1658</v>
@@ -2573,7 +2573,7 @@
         <v>3</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I40" s="5" t="n">
         <v>2487</v>
@@ -2765,7 +2765,7 @@
         <v>2</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I44" s="5" t="n">
         <v>1658</v>
@@ -2813,7 +2813,7 @@
         <v>2</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I45" s="5" t="n">
         <v>1658</v>
@@ -3053,7 +3053,7 @@
         <v>4</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>44000</v>
+        <v>38700</v>
       </c>
       <c r="I50" s="5" t="n">
         <v>3193</v>
@@ -3245,7 +3245,7 @@
         <v>2</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I54" s="5" t="n">
         <v>4743</v>
@@ -3293,7 +3293,7 @@
         <v>5</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I55" s="5" t="n">
         <v>3991</v>
@@ -3389,7 +3389,7 @@
         <v>2</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I57" s="5" t="n">
         <v>4743</v>
@@ -3677,7 +3677,7 @@
         <v>5</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>135500</v>
+        <v>129875</v>
       </c>
       <c r="I63" s="5" t="n">
         <v>11689</v>
@@ -3725,7 +3725,7 @@
         <v>4</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I64" s="5" t="n">
         <v>9351</v>
@@ -3773,7 +3773,7 @@
         <v>2</v>
       </c>
       <c r="H65" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I65" s="5" t="n">
         <v>4743</v>
@@ -3869,7 +3869,7 @@
         <v>2</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I67" s="5" t="n">
         <v>1658</v>
@@ -4157,7 +4157,7 @@
         <v>2</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I73" s="5" t="n">
         <v>4743</v>
@@ -4685,7 +4685,7 @@
         <v>2</v>
       </c>
       <c r="H84" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I84" s="5" t="n">
         <v>4743</v>
@@ -4829,7 +4829,7 @@
         <v>2</v>
       </c>
       <c r="H87" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I87" s="5" t="n">
         <v>1658</v>
@@ -4973,7 +4973,7 @@
         <v>3</v>
       </c>
       <c r="H90" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I90" s="5" t="n">
         <v>7115</v>
@@ -5453,7 +5453,7 @@
         <v>96</v>
       </c>
       <c r="H100" s="5" t="n">
-        <v>2601600</v>
+        <v>2481600</v>
       </c>
       <c r="I100" s="5" t="n">
         <v>223344</v>
@@ -5501,7 +5501,7 @@
         <v>2</v>
       </c>
       <c r="H101" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I101" s="5" t="n">
         <v>4743</v>
@@ -5645,7 +5645,7 @@
         <v>7</v>
       </c>
       <c r="H104" s="5" t="n">
-        <v>77000</v>
+        <v>66850</v>
       </c>
       <c r="I104" s="5" t="n">
         <v>5515</v>
@@ -5837,7 +5837,7 @@
         <v>4</v>
       </c>
       <c r="H108" s="5" t="n">
-        <v>44000</v>
+        <v>38700</v>
       </c>
       <c r="I108" s="5" t="n">
         <v>3193</v>
@@ -5885,7 +5885,7 @@
         <v>7</v>
       </c>
       <c r="H109" s="5" t="n">
-        <v>189700</v>
+        <v>180950</v>
       </c>
       <c r="I109" s="5" t="n">
         <v>16286</v>
@@ -5933,7 +5933,7 @@
         <v>17</v>
       </c>
       <c r="H110" s="5" t="n">
-        <v>460700</v>
+        <v>439450</v>
       </c>
       <c r="I110" s="5" t="n">
         <v>39551</v>
@@ -6029,7 +6029,7 @@
         <v>3</v>
       </c>
       <c r="H112" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I112" s="5" t="n">
         <v>7115</v>
@@ -6077,7 +6077,7 @@
         <v>2</v>
       </c>
       <c r="H113" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I113" s="5" t="n">
         <v>4743</v>
@@ -6269,7 +6269,7 @@
         <v>2</v>
       </c>
       <c r="H117" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I117" s="5" t="n">
         <v>4743</v>
@@ -6989,7 +6989,7 @@
         <v>2</v>
       </c>
       <c r="H132" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I132" s="5" t="n">
         <v>4743</v>
@@ -7181,7 +7181,7 @@
         <v>2</v>
       </c>
       <c r="H136" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I136" s="5" t="n">
         <v>4743</v>
@@ -7325,7 +7325,7 @@
         <v>2</v>
       </c>
       <c r="H139" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I139" s="5" t="n">
         <v>1658</v>
@@ -7469,7 +7469,7 @@
         <v>3</v>
       </c>
       <c r="H142" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I142" s="5" t="n">
         <v>7115</v>
@@ -7709,7 +7709,7 @@
         <v>5</v>
       </c>
       <c r="H147" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I147" s="5" t="n">
         <v>3991</v>
@@ -7805,7 +7805,7 @@
         <v>6</v>
       </c>
       <c r="H149" s="5" t="n">
-        <v>40200</v>
+        <v>32700</v>
       </c>
       <c r="I149" s="5" t="n">
         <v>2943</v>
@@ -7853,7 +7853,7 @@
         <v>5</v>
       </c>
       <c r="H150" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I150" s="5" t="n">
         <v>3991</v>
@@ -8093,7 +8093,7 @@
         <v>4</v>
       </c>
       <c r="H155" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I155" s="5" t="n">
         <v>9351</v>
@@ -8141,7 +8141,7 @@
         <v>6</v>
       </c>
       <c r="H156" s="5" t="n">
-        <v>66000</v>
+        <v>57300</v>
       </c>
       <c r="I156" s="5" t="n">
         <v>4727</v>
@@ -8381,7 +8381,7 @@
         <v>20</v>
       </c>
       <c r="H161" s="5" t="n">
-        <v>542000</v>
+        <v>517000</v>
       </c>
       <c r="I161" s="5" t="n">
         <v>46530</v>
@@ -8765,7 +8765,7 @@
         <v>3</v>
       </c>
       <c r="H169" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I169" s="5" t="n">
         <v>7115</v>
@@ -8861,7 +8861,7 @@
         <v>2</v>
       </c>
       <c r="H171" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I171" s="5" t="n">
         <v>1658</v>
@@ -9197,7 +9197,7 @@
         <v>2</v>
       </c>
       <c r="H178" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I178" s="5" t="n">
         <v>1658</v>
@@ -9485,7 +9485,7 @@
         <v>2</v>
       </c>
       <c r="H184" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I184" s="5" t="n">
         <v>4743</v>
@@ -9533,7 +9533,7 @@
         <v>2</v>
       </c>
       <c r="H185" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I185" s="5" t="n">
         <v>1658</v>
@@ -9581,7 +9581,7 @@
         <v>3</v>
       </c>
       <c r="H186" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I186" s="5" t="n">
         <v>7115</v>
@@ -9725,7 +9725,7 @@
         <v>5</v>
       </c>
       <c r="H189" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I189" s="5" t="n">
         <v>3991</v>
@@ -9773,7 +9773,7 @@
         <v>2</v>
       </c>
       <c r="H190" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I190" s="5" t="n">
         <v>1658</v>
@@ -10013,7 +10013,7 @@
         <v>24</v>
       </c>
       <c r="H195" s="5" t="n">
-        <v>650400</v>
+        <v>620400</v>
       </c>
       <c r="I195" s="5" t="n">
         <v>55836</v>
@@ -10109,7 +10109,7 @@
         <v>12</v>
       </c>
       <c r="H197" s="5" t="n">
-        <v>325200</v>
+        <v>310200</v>
       </c>
       <c r="I197" s="5" t="n">
         <v>27918</v>
@@ -10157,7 +10157,7 @@
         <v>6</v>
       </c>
       <c r="H198" s="5" t="n">
-        <v>40200</v>
+        <v>32700</v>
       </c>
       <c r="I198" s="5" t="n">
         <v>2943</v>
@@ -10253,7 +10253,7 @@
         <v>8</v>
       </c>
       <c r="H200" s="5" t="n">
-        <v>88000</v>
+        <v>76400</v>
       </c>
       <c r="I200" s="5" t="n">
         <v>6303</v>
@@ -10301,7 +10301,7 @@
         <v>5</v>
       </c>
       <c r="H201" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I201" s="5" t="n">
         <v>3991</v>
@@ -10397,7 +10397,7 @@
         <v>2</v>
       </c>
       <c r="H203" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I203" s="5" t="n">
         <v>4743</v>
@@ -10445,7 +10445,7 @@
         <v>10</v>
       </c>
       <c r="H204" s="5" t="n">
-        <v>271000</v>
+        <v>258500</v>
       </c>
       <c r="I204" s="5" t="n">
         <v>23265</v>
@@ -10589,7 +10589,7 @@
         <v>6</v>
       </c>
       <c r="H207" s="5" t="n">
-        <v>162600</v>
+        <v>155100</v>
       </c>
       <c r="I207" s="5" t="n">
         <v>13959</v>
@@ -10733,7 +10733,7 @@
         <v>2</v>
       </c>
       <c r="H210" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I210" s="5" t="n">
         <v>4743</v>
@@ -10829,7 +10829,7 @@
         <v>12</v>
       </c>
       <c r="H212" s="5" t="n">
-        <v>325200</v>
+        <v>310200</v>
       </c>
       <c r="I212" s="5" t="n">
         <v>27918</v>
@@ -10925,7 +10925,7 @@
         <v>2</v>
       </c>
       <c r="H214" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I214" s="5" t="n">
         <v>1658</v>
@@ -11021,7 +11021,7 @@
         <v>2</v>
       </c>
       <c r="H216" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I216" s="5" t="n">
         <v>4743</v>
@@ -11741,7 +11741,7 @@
         <v>4</v>
       </c>
       <c r="H231" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I231" s="5" t="n">
         <v>9351</v>
@@ -11789,7 +11789,7 @@
         <v>3</v>
       </c>
       <c r="H232" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I232" s="5" t="n">
         <v>2487</v>
@@ -11837,7 +11837,7 @@
         <v>5</v>
       </c>
       <c r="H233" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I233" s="5" t="n">
         <v>3991</v>
@@ -11933,7 +11933,7 @@
         <v>3</v>
       </c>
       <c r="H235" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I235" s="5" t="n">
         <v>2487</v>
@@ -11981,7 +11981,7 @@
         <v>2</v>
       </c>
       <c r="H236" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I236" s="5" t="n">
         <v>1658</v>
@@ -12029,7 +12029,7 @@
         <v>4</v>
       </c>
       <c r="H237" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I237" s="5" t="n">
         <v>9351</v>
@@ -12173,7 +12173,7 @@
         <v>2</v>
       </c>
       <c r="H240" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I240" s="5" t="n">
         <v>1658</v>
@@ -12317,7 +12317,7 @@
         <v>2</v>
       </c>
       <c r="H243" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I243" s="5" t="n">
         <v>1658</v>
@@ -12605,7 +12605,7 @@
         <v>24</v>
       </c>
       <c r="H249" s="5" t="n">
-        <v>564600</v>
+        <v>542100</v>
       </c>
       <c r="I249" s="5" t="n">
         <v>48789</v>
@@ -12653,7 +12653,7 @@
         <v>2</v>
       </c>
       <c r="H250" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I250" s="5" t="n">
         <v>1658</v>
@@ -12797,7 +12797,7 @@
         <v>6</v>
       </c>
       <c r="H253" s="5" t="n">
-        <v>162600</v>
+        <v>155100</v>
       </c>
       <c r="I253" s="5" t="n">
         <v>13959</v>
@@ -12893,7 +12893,7 @@
         <v>3</v>
       </c>
       <c r="H255" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I255" s="5" t="n">
         <v>2487</v>
@@ -13469,7 +13469,7 @@
         <v>3</v>
       </c>
       <c r="H267" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I267" s="5" t="n">
         <v>2487</v>
@@ -13661,7 +13661,7 @@
         <v>3</v>
       </c>
       <c r="H271" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I271" s="5" t="n">
         <v>7115</v>
@@ -13709,7 +13709,7 @@
         <v>4</v>
       </c>
       <c r="H272" s="5" t="n">
-        <v>44000</v>
+        <v>38700</v>
       </c>
       <c r="I272" s="5" t="n">
         <v>3193</v>
@@ -13901,7 +13901,7 @@
         <v>5</v>
       </c>
       <c r="H276" s="5" t="n">
-        <v>55000</v>
+        <v>48375</v>
       </c>
       <c r="I276" s="5" t="n">
         <v>3991</v>
@@ -13949,7 +13949,7 @@
         <v>2</v>
       </c>
       <c r="H277" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I277" s="5" t="n">
         <v>1658</v>
@@ -14045,7 +14045,7 @@
         <v>2</v>
       </c>
       <c r="H279" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I279" s="5" t="n">
         <v>1658</v>
@@ -14093,7 +14093,7 @@
         <v>2</v>
       </c>
       <c r="H280" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I280" s="5" t="n">
         <v>4743</v>
@@ -14141,7 +14141,7 @@
         <v>2</v>
       </c>
       <c r="H281" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I281" s="5" t="n">
         <v>1658</v>
@@ -14237,7 +14237,7 @@
         <v>2</v>
       </c>
       <c r="H283" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I283" s="5" t="n">
         <v>1658</v>
@@ -14285,7 +14285,7 @@
         <v>18</v>
       </c>
       <c r="H284" s="5" t="n">
-        <v>198000</v>
+        <v>171900</v>
       </c>
       <c r="I284" s="5" t="n">
         <v>14182</v>
@@ -14429,7 +14429,7 @@
         <v>2</v>
       </c>
       <c r="H287" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I287" s="5" t="n">
         <v>1658</v>
@@ -14621,7 +14621,7 @@
         <v>16</v>
       </c>
       <c r="H291" s="5" t="n">
-        <v>433600</v>
+        <v>413600</v>
       </c>
       <c r="I291" s="5" t="n">
         <v>37224</v>
@@ -15293,7 +15293,7 @@
         <v>2</v>
       </c>
       <c r="H305" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I305" s="5" t="n">
         <v>1658</v>
@@ -15389,7 +15389,7 @@
         <v>10</v>
       </c>
       <c r="H307" s="5" t="n">
-        <v>110000</v>
+        <v>95500</v>
       </c>
       <c r="I307" s="5" t="n">
         <v>7879</v>
@@ -15533,7 +15533,7 @@
         <v>3</v>
       </c>
       <c r="H310" s="5" t="n">
-        <v>28700</v>
+        <v>26800</v>
       </c>
       <c r="I310" s="5" t="n">
         <v>2261</v>
@@ -15581,7 +15581,7 @@
         <v>2</v>
       </c>
       <c r="H311" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I311" s="5" t="n">
         <v>4743</v>
@@ -15629,7 +15629,7 @@
         <v>2</v>
       </c>
       <c r="H312" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I312" s="5" t="n">
         <v>1658</v>
@@ -15773,7 +15773,7 @@
         <v>2</v>
       </c>
       <c r="H315" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I315" s="5" t="n">
         <v>1658</v>
@@ -15821,7 +15821,7 @@
         <v>6</v>
       </c>
       <c r="H316" s="5" t="n">
-        <v>162600</v>
+        <v>155100</v>
       </c>
       <c r="I316" s="5" t="n">
         <v>13959</v>
@@ -15965,7 +15965,7 @@
         <v>2</v>
       </c>
       <c r="H319" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I319" s="5" t="n">
         <v>1658</v>
@@ -16013,7 +16013,7 @@
         <v>2</v>
       </c>
       <c r="H320" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I320" s="5" t="n">
         <v>1658</v>
@@ -16061,7 +16061,7 @@
         <v>3</v>
       </c>
       <c r="H321" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I321" s="5" t="n">
         <v>2487</v>
@@ -16157,7 +16157,7 @@
         <v>3</v>
       </c>
       <c r="H323" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I323" s="5" t="n">
         <v>2487</v>
@@ -16253,7 +16253,7 @@
         <v>2</v>
       </c>
       <c r="H325" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I325" s="5" t="n">
         <v>1658</v>
@@ -16349,7 +16349,7 @@
         <v>2</v>
       </c>
       <c r="H327" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I327" s="5" t="n">
         <v>1658</v>
@@ -16397,7 +16397,7 @@
         <v>24</v>
       </c>
       <c r="H328" s="5" t="n">
-        <v>264000</v>
+        <v>229200</v>
       </c>
       <c r="I328" s="5" t="n">
         <v>18909</v>
@@ -16445,7 +16445,7 @@
         <v>24</v>
       </c>
       <c r="H329" s="5" t="n">
-        <v>264000</v>
+        <v>229200</v>
       </c>
       <c r="I329" s="5" t="n">
         <v>18909</v>
@@ -16493,7 +16493,7 @@
         <v>4</v>
       </c>
       <c r="H330" s="5" t="n">
-        <v>44000</v>
+        <v>38700</v>
       </c>
       <c r="I330" s="5" t="n">
         <v>3193</v>
@@ -16541,7 +16541,7 @@
         <v>2</v>
       </c>
       <c r="H331" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I331" s="5" t="n">
         <v>1658</v>
@@ -16637,7 +16637,7 @@
         <v>2</v>
       </c>
       <c r="H333" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I333" s="5" t="n">
         <v>4743</v>
@@ -16781,7 +16781,7 @@
         <v>2</v>
       </c>
       <c r="H336" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I336" s="5" t="n">
         <v>1658</v>
@@ -16829,7 +16829,7 @@
         <v>2</v>
       </c>
       <c r="H337" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I337" s="5" t="n">
         <v>1658</v>
@@ -16877,7 +16877,7 @@
         <v>2</v>
       </c>
       <c r="H338" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I338" s="5" t="n">
         <v>1658</v>
@@ -17021,7 +17021,7 @@
         <v>7</v>
       </c>
       <c r="H341" s="5" t="n">
-        <v>77000</v>
+        <v>66850</v>
       </c>
       <c r="I341" s="5" t="n">
         <v>5515</v>
@@ -17117,7 +17117,7 @@
         <v>12</v>
       </c>
       <c r="H343" s="5" t="n">
-        <v>325200</v>
+        <v>310200</v>
       </c>
       <c r="I343" s="5" t="n">
         <v>27918</v>
@@ -17165,7 +17165,7 @@
         <v>2</v>
       </c>
       <c r="H344" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I344" s="5" t="n">
         <v>1658</v>
@@ -17405,7 +17405,7 @@
         <v>5</v>
       </c>
       <c r="H349" s="5" t="n">
-        <v>135500</v>
+        <v>129875</v>
       </c>
       <c r="I349" s="5" t="n">
         <v>11689</v>
@@ -17501,7 +17501,7 @@
         <v>6</v>
       </c>
       <c r="H351" s="5" t="n">
-        <v>162600</v>
+        <v>155100</v>
       </c>
       <c r="I351" s="5" t="n">
         <v>13959</v>
@@ -17549,7 +17549,7 @@
         <v>50</v>
       </c>
       <c r="H352" s="5" t="n">
-        <v>1355000</v>
+        <v>1292500</v>
       </c>
       <c r="I352" s="5" t="n">
         <v>116325</v>
@@ -17933,7 +17933,7 @@
         <v>10</v>
       </c>
       <c r="H360" s="5" t="n">
-        <v>271000</v>
+        <v>258500</v>
       </c>
       <c r="I360" s="5" t="n">
         <v>23265</v>
@@ -18029,7 +18029,7 @@
         <v>4</v>
       </c>
       <c r="H362" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I362" s="5" t="n">
         <v>9351</v>
@@ -18125,7 +18125,7 @@
         <v>15</v>
       </c>
       <c r="H364" s="5" t="n">
-        <v>406500</v>
+        <v>387750</v>
       </c>
       <c r="I364" s="5" t="n">
         <v>34898</v>
@@ -18221,7 +18221,7 @@
         <v>10</v>
       </c>
       <c r="H366" s="5" t="n">
-        <v>271000</v>
+        <v>258500</v>
       </c>
       <c r="I366" s="5" t="n">
         <v>23265</v>
@@ -18365,7 +18365,7 @@
         <v>20</v>
       </c>
       <c r="H369" s="5" t="n">
-        <v>542000</v>
+        <v>517000</v>
       </c>
       <c r="I369" s="5" t="n">
         <v>46530</v>
@@ -18605,7 +18605,7 @@
         <v>72</v>
       </c>
       <c r="H374" s="5" t="n">
-        <v>1951200</v>
+        <v>1861200</v>
       </c>
       <c r="I374" s="5" t="n">
         <v>167508</v>
@@ -18749,7 +18749,7 @@
         <v>4</v>
       </c>
       <c r="H377" s="5" t="n">
-        <v>108400</v>
+        <v>103900</v>
       </c>
       <c r="I377" s="5" t="n">
         <v>9351</v>
@@ -19037,7 +19037,7 @@
         <v>2</v>
       </c>
       <c r="H383" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I383" s="5" t="n">
         <v>4743</v>
@@ -19565,7 +19565,7 @@
         <v>4</v>
       </c>
       <c r="H394" s="5" t="n">
-        <v>69000</v>
+        <v>67500</v>
       </c>
       <c r="I394" s="5" t="n">
         <v>6075</v>
@@ -19901,7 +19901,7 @@
         <v>12</v>
       </c>
       <c r="H401" s="5" t="n">
-        <v>325200</v>
+        <v>310200</v>
       </c>
       <c r="I401" s="5" t="n">
         <v>27918</v>
@@ -20093,7 +20093,7 @@
         <v>2</v>
       </c>
       <c r="H405" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I405" s="5" t="n">
         <v>4743</v>
@@ -20477,7 +20477,7 @@
         <v>3</v>
       </c>
       <c r="H413" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I413" s="5" t="n">
         <v>7115</v>
@@ -20525,7 +20525,7 @@
         <v>2</v>
       </c>
       <c r="H414" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I414" s="5" t="n">
         <v>4743</v>
@@ -20621,7 +20621,7 @@
         <v>24</v>
       </c>
       <c r="H416" s="5" t="n">
-        <v>650400</v>
+        <v>620400</v>
       </c>
       <c r="I416" s="5" t="n">
         <v>55836</v>
@@ -20813,7 +20813,7 @@
         <v>2</v>
       </c>
       <c r="H420" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I420" s="5" t="n">
         <v>4743</v>
@@ -20957,7 +20957,7 @@
         <v>2</v>
       </c>
       <c r="H423" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I423" s="5" t="n">
         <v>1658</v>
@@ -21629,7 +21629,7 @@
         <v>2</v>
       </c>
       <c r="H437" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I437" s="5" t="n">
         <v>4743</v>
@@ -21773,7 +21773,7 @@
         <v>2</v>
       </c>
       <c r="H440" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I440" s="5" t="n">
         <v>1658</v>
@@ -21917,7 +21917,7 @@
         <v>25</v>
       </c>
       <c r="H443" s="5" t="n">
-        <v>677500</v>
+        <v>646250</v>
       </c>
       <c r="I443" s="5" t="n">
         <v>58163</v>
@@ -21965,7 +21965,7 @@
         <v>2</v>
       </c>
       <c r="H444" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I444" s="5" t="n">
         <v>1658</v>
@@ -22109,7 +22109,7 @@
         <v>2</v>
       </c>
       <c r="H447" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I447" s="5" t="n">
         <v>4743</v>
@@ -22205,7 +22205,7 @@
         <v>2</v>
       </c>
       <c r="H449" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I449" s="5" t="n">
         <v>1658</v>
@@ -22397,7 +22397,7 @@
         <v>3</v>
       </c>
       <c r="H453" s="5" t="n">
-        <v>33000</v>
+        <v>30150</v>
       </c>
       <c r="I453" s="5" t="n">
         <v>2487</v>
@@ -22445,7 +22445,7 @@
         <v>2</v>
       </c>
       <c r="H454" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I454" s="5" t="n">
         <v>1658</v>
@@ -22541,7 +22541,7 @@
         <v>2</v>
       </c>
       <c r="H456" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I456" s="5" t="n">
         <v>1658</v>
@@ -22733,7 +22733,7 @@
         <v>15</v>
       </c>
       <c r="H460" s="5" t="n">
-        <v>406500</v>
+        <v>387750</v>
       </c>
       <c r="I460" s="5" t="n">
         <v>34898</v>
@@ -22781,7 +22781,7 @@
         <v>2</v>
       </c>
       <c r="H461" s="5" t="n">
-        <v>54200</v>
+        <v>52700</v>
       </c>
       <c r="I461" s="5" t="n">
         <v>4743</v>
@@ -22925,7 +22925,7 @@
         <v>7</v>
       </c>
       <c r="H464" s="5" t="n">
-        <v>77000</v>
+        <v>66850</v>
       </c>
       <c r="I464" s="5" t="n">
         <v>5515</v>
@@ -22973,7 +22973,7 @@
         <v>2</v>
       </c>
       <c r="H465" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I465" s="5" t="n">
         <v>1658</v>
@@ -23069,7 +23069,7 @@
         <v>2</v>
       </c>
       <c r="H467" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I467" s="5" t="n">
         <v>1658</v>
@@ -23405,7 +23405,7 @@
         <v>10</v>
       </c>
       <c r="H474" s="5" t="n">
-        <v>271000</v>
+        <v>258500</v>
       </c>
       <c r="I474" s="5" t="n">
         <v>23265</v>
@@ -23453,7 +23453,7 @@
         <v>3</v>
       </c>
       <c r="H475" s="5" t="n">
-        <v>81300</v>
+        <v>79050</v>
       </c>
       <c r="I475" s="5" t="n">
         <v>7115</v>
@@ -23549,7 +23549,7 @@
         <v>2</v>
       </c>
       <c r="H477" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I477" s="5" t="n">
         <v>1658</v>
@@ -23645,7 +23645,7 @@
         <v>2</v>
       </c>
       <c r="H479" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I479" s="5" t="n">
         <v>1658</v>
@@ -23693,7 +23693,7 @@
         <v>2</v>
       </c>
       <c r="H480" s="5" t="n">
-        <v>22000</v>
+        <v>20100</v>
       </c>
       <c r="I480" s="5" t="n">
         <v>1658</v>
@@ -23741,7 +23741,7 @@
         <v>4</v>
       </c>
       <c r="H481" s="5" t="n">
-        <v>44000</v>
+        <v>38700</v>
       </c>
       <c r="I481" s="5" t="n">
         <v>3193</v>
@@ -24243,7 +24243,7 @@
         </is>
       </c>
       <c r="H492" s="9" t="n">
-        <v>34178600</v>
+        <v>32854750</v>
       </c>
       <c r="I492" s="9" t="n">
         <v>2930575</v>
@@ -25189,19 +25189,19 @@
         <v>3</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>27100</v>
+        <v>26350</v>
       </c>
       <c r="I32" s="5" t="n">
         <v>2372</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>8.752767527675278</v>
+        <v>9.001897533206831</v>
       </c>
       <c r="K32" s="5" t="n">
         <v>1318</v>
       </c>
       <c r="L32" s="10" t="n">
-        <v>4.863468634686347</v>
+        <v>5.001897533206831</v>
       </c>
       <c r="M32" s="5" t="n">
         <v>417</v>
@@ -25508,19 +25508,19 @@
         <v>58</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>27100</v>
+        <v>26350</v>
       </c>
       <c r="I41" s="5" t="n">
         <v>2372</v>
       </c>
       <c r="J41" s="10" t="n">
-        <v>8.752767527675278</v>
+        <v>9.001897533206831</v>
       </c>
       <c r="K41" s="5" t="n">
         <v>1318</v>
       </c>
       <c r="L41" s="10" t="n">
-        <v>4.863468634686347</v>
+        <v>5.001897533206831</v>
       </c>
       <c r="M41" s="5" t="n">
         <v>577</v>
@@ -25571,19 +25571,19 @@
         <v>51</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>27100</v>
+        <v>25975</v>
       </c>
       <c r="I42" s="5" t="n">
         <v>2338</v>
       </c>
       <c r="J42" s="10" t="n">
-        <v>8.627306273062731</v>
+        <v>9.000962463907603</v>
       </c>
       <c r="K42" s="5" t="n">
         <v>1299</v>
       </c>
       <c r="L42" s="10" t="n">
-        <v>4.793357933579336</v>
+        <v>5.000962463907603</v>
       </c>
       <c r="M42" s="5" t="n">
         <v>297</v>
@@ -25634,19 +25634,19 @@
         <v>538</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>27100</v>
+        <v>25896</v>
       </c>
       <c r="I43" s="5" t="n">
         <v>2331</v>
       </c>
       <c r="J43" s="10" t="n">
-        <v>8.601476014760149</v>
+        <v>9.001390176088972</v>
       </c>
       <c r="K43" s="5" t="n">
         <v>1295</v>
       </c>
       <c r="L43" s="10" t="n">
-        <v>4.778597785977859</v>
+        <v>5.000772320049428</v>
       </c>
       <c r="M43" s="5" t="n">
         <v>101</v>
@@ -26018,19 +26018,19 @@
         <v>4</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>27100</v>
+        <v>26350</v>
       </c>
       <c r="I55" s="5" t="n">
         <v>2372</v>
       </c>
       <c r="J55" s="10" t="n">
-        <v>8.752767527675278</v>
+        <v>9.001897533206831</v>
       </c>
       <c r="K55" s="5" t="n">
         <v>1318</v>
       </c>
       <c r="L55" s="10" t="n">
-        <v>4.863468634686347</v>
+        <v>5.001897533206831</v>
       </c>
       <c r="M55" s="5" t="n">
         <v>625</v>
@@ -26339,19 +26339,19 @@
         <v>27</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>11000</v>
+        <v>10050</v>
       </c>
       <c r="I66" s="5" t="n">
         <v>829</v>
       </c>
       <c r="J66" s="10" t="n">
-        <v>7.536363636363637</v>
+        <v>8.248756218905474</v>
       </c>
       <c r="K66" s="5" t="n">
         <v>452</v>
       </c>
       <c r="L66" s="10" t="n">
-        <v>4.109090909090908</v>
+        <v>4.497512437810945</v>
       </c>
       <c r="M66" s="5" t="n">
         <v>609</v>
@@ -26402,19 +26402,19 @@
         <v>12</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>11000</v>
+        <v>9675</v>
       </c>
       <c r="I67" s="5" t="n">
         <v>798</v>
       </c>
       <c r="J67" s="10" t="n">
-        <v>7.254545454545455</v>
+        <v>8.248062015503876</v>
       </c>
       <c r="K67" s="5" t="n">
         <v>436</v>
       </c>
       <c r="L67" s="10" t="n">
-        <v>3.963636363636364</v>
+        <v>4.506459948320414</v>
       </c>
       <c r="M67" s="5" t="n">
         <v>313</v>
@@ -26465,19 +26465,19 @@
         <v>14</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>11000</v>
+        <v>9550</v>
       </c>
       <c r="I68" s="5" t="n">
         <v>788</v>
       </c>
       <c r="J68" s="10" t="n">
-        <v>7.163636363636364</v>
+        <v>8.25130890052356</v>
       </c>
       <c r="K68" s="5" t="n">
         <v>430</v>
       </c>
       <c r="L68" s="10" t="n">
-        <v>3.909090909090909</v>
+        <v>4.502617801047121</v>
       </c>
       <c r="M68" s="5" t="n">
         <v>179</v>
@@ -26593,19 +26593,19 @@
         <v>54</v>
       </c>
       <c r="H72" s="5" t="n">
-        <v>11000</v>
+        <v>10050</v>
       </c>
       <c r="I72" s="5" t="n">
         <v>829</v>
       </c>
       <c r="J72" s="10" t="n">
-        <v>7.536363636363637</v>
+        <v>8.248756218905474</v>
       </c>
       <c r="K72" s="5" t="n">
         <v>452</v>
       </c>
       <c r="L72" s="10" t="n">
-        <v>4.109090909090908</v>
+        <v>4.497512437810945</v>
       </c>
       <c r="M72" s="5" t="n">
         <v>573</v>
@@ -26656,19 +26656,19 @@
         <v>23</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>11000</v>
+        <v>9675</v>
       </c>
       <c r="I73" s="5" t="n">
         <v>798</v>
       </c>
       <c r="J73" s="10" t="n">
-        <v>7.254545454545455</v>
+        <v>8.248062015503876</v>
       </c>
       <c r="K73" s="5" t="n">
         <v>435</v>
       </c>
       <c r="L73" s="10" t="n">
-        <v>3.954545454545454</v>
+        <v>4.496124031007752</v>
       </c>
       <c r="M73" s="5" t="n">
         <v>275</v>
@@ -26719,19 +26719,19 @@
         <v>72</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>11000</v>
+        <v>9550</v>
       </c>
       <c r="I74" s="5" t="n">
         <v>788</v>
       </c>
       <c r="J74" s="10" t="n">
-        <v>7.163636363636364</v>
+        <v>8.25130890052356</v>
       </c>
       <c r="K74" s="5" t="n">
         <v>430</v>
       </c>
       <c r="L74" s="10" t="n">
-        <v>3.909090909090909</v>
+        <v>4.502617801047121</v>
       </c>
       <c r="M74" s="5" t="n">
         <v>119</v>
@@ -27042,19 +27042,19 @@
         <v>6</v>
       </c>
       <c r="H87" s="5" t="n">
-        <v>6700</v>
+        <v>5450</v>
       </c>
       <c r="I87" s="5" t="n">
         <v>491</v>
       </c>
       <c r="J87" s="10" t="n">
-        <v>7.328358208955224</v>
+        <v>9.009174311926605</v>
       </c>
       <c r="K87" s="5" t="n">
         <v>300</v>
       </c>
       <c r="L87" s="10" t="n">
-        <v>4.477611940298507</v>
+        <v>5.504587155963304</v>
       </c>
       <c r="M87" s="5" t="n">
         <v>208</v>
@@ -27107,19 +27107,19 @@
         <v>6</v>
       </c>
       <c r="H90" s="5" t="n">
-        <v>6700</v>
+        <v>5450</v>
       </c>
       <c r="I90" s="5" t="n">
         <v>491</v>
       </c>
       <c r="J90" s="10" t="n">
-        <v>7.328358208955224</v>
+        <v>9.009174311926605</v>
       </c>
       <c r="K90" s="5" t="n">
         <v>300</v>
       </c>
       <c r="L90" s="10" t="n">
-        <v>4.477611940298507</v>
+        <v>5.504587155963304</v>
       </c>
       <c r="M90" s="5" t="n">
         <v>208</v>
@@ -27218,23 +27218,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HARGA MODAL PER PRODUK</t>
+          <t>CARA HITUNG HARGA MODAL &amp; HARGA MARKETPLACE</t>
         </is>
       </c>
     </row>
@@ -27248,7 +27249,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rumus: Harga Beli/Karton (in PPN) / Pcs per Karton = Harga Beli/unit. + Margin 3% = Harga Modal/unit.</t>
+          <t>Rumus: Beli (in PPN) + Margin 3% = Harga Modal. Lalu Modal / (1 - 18% biaya platform) = Harga Marketplace.</t>
         </is>
       </c>
     </row>
@@ -27271,27 +27272,32 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Satuan Jual</t>
+          <t>Pcs/Karton</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Pcs/Karton</t>
+          <t>Beli/Karton in PPN (Rp)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Harga Beli/Karton in PPN (Rp)</t>
+          <t>Beli/unit (Rp)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Harga Beli/unit (Rp)</t>
+          <t>Modal/Karton +3% (Rp)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Harga Modal/unit +3% (Rp)</t>
+          <t>Modal/unit +3% (Rp)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Harga Marketplace (Rp) (referensi)</t>
         </is>
       </c>
     </row>
@@ -27309,22 +27315,23 @@
           <t>Autan Care Protect Sachet 6ml-1152ID</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>renceng</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>1152</v>
       </c>
+      <c r="E6" s="5" t="n">
+        <v>460643</v>
+      </c>
       <c r="F6" s="5" t="n">
-        <v>460643</v>
+        <v>400</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>400</v>
+        <v>474462</v>
       </c>
       <c r="H6" s="5" t="n">
         <v>412</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>6100</v>
       </c>
     </row>
     <row r="7">
@@ -27341,22 +27348,23 @@
           <t>AUTAN SAKURA SACHET 6ml.1152ID</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>renceng</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>1152</v>
       </c>
+      <c r="E7" s="5" t="n">
+        <v>460643</v>
+      </c>
       <c r="F7" s="5" t="n">
-        <v>460643</v>
+        <v>400</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>400</v>
+        <v>474462</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>412</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>6100</v>
       </c>
     </row>
     <row r="8">
@@ -27373,22 +27381,23 @@
           <t>Autan All Night Tube 50ml.144ID</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E8" s="5" t="n">
+        <v>1369075</v>
+      </c>
       <c r="F8" s="5" t="n">
-        <v>1369075</v>
+        <v>9507</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>9507</v>
+        <v>1410147</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>9793</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="9">
@@ -27405,22 +27414,23 @@
           <t>AUTAN SAKURA TUBE 50ML.144 ID</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E9" s="5" t="n">
+        <v>1369075</v>
+      </c>
       <c r="F9" s="5" t="n">
-        <v>1369075</v>
+        <v>9507</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>9507</v>
+        <v>1410147</v>
       </c>
       <c r="H9" s="5" t="n">
         <v>9793</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="10">
@@ -27437,22 +27447,23 @@
           <t>Autan Care Protect Tube 50ml-144ID</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
+      <c r="D10" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E10" s="5" t="n">
+        <v>1369075</v>
+      </c>
       <c r="F10" s="5" t="n">
-        <v>1369075</v>
+        <v>9507</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>9507</v>
+        <v>1410147</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>9793</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="11">
@@ -27469,22 +27480,23 @@
           <t>Autan Floral Protect Tube 50ml.144ID</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
+      <c r="D11" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E11" s="5" t="n">
+        <v>1369075</v>
+      </c>
       <c r="F11" s="5" t="n">
-        <v>1369075</v>
+        <v>9507</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>9507</v>
+        <v>1410147</v>
       </c>
       <c r="H11" s="5" t="n">
         <v>9793</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>12000</v>
       </c>
     </row>
     <row r="12">
@@ -27501,22 +27513,23 @@
           <t>AUTAN RFSH SPRITZ LIQ BT 100ML-144ID</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E12" s="5" t="n">
+        <v>1829712</v>
+      </c>
       <c r="F12" s="5" t="n">
-        <v>1829712</v>
+        <v>12706</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>12706</v>
+        <v>1884604</v>
       </c>
       <c r="H12" s="5" t="n">
         <v>13088</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>16000</v>
       </c>
     </row>
     <row r="13">
@@ -27533,22 +27546,23 @@
           <t>Kiwi Paste SP Neutral 45ml-48ID</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="E13" s="5" t="n">
+        <v>1001942</v>
+      </c>
       <c r="F13" s="5" t="n">
-        <v>1001942</v>
+        <v>20874</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>20874</v>
+        <v>1032000</v>
       </c>
       <c r="H13" s="5" t="n">
         <v>21500</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>26300</v>
       </c>
     </row>
     <row r="14">
@@ -27565,22 +27579,23 @@
           <t>Kiwi Paste SP Brown 17.5ml-144ID</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>144</v>
       </c>
+      <c r="E14" s="5" t="n">
+        <v>1322563</v>
+      </c>
       <c r="F14" s="5" t="n">
-        <v>1322563</v>
+        <v>9184</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>9184</v>
+        <v>1362240</v>
       </c>
       <c r="H14" s="5" t="n">
         <v>9460</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>11600</v>
       </c>
     </row>
     <row r="15">
@@ -27597,22 +27612,23 @@
           <t>Kiwi Paste SP Black 45ml-48 ID</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
+      <c r="D15" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="E15" s="5" t="n">
+        <v>1001942</v>
+      </c>
       <c r="F15" s="5" t="n">
-        <v>1001942</v>
+        <v>20874</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>20874</v>
+        <v>1032000</v>
       </c>
       <c r="H15" s="5" t="n">
         <v>21500</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>26300</v>
       </c>
     </row>
     <row r="16">
@@ -27629,22 +27645,23 @@
           <t>Kiwi Wax Rich SP Brown 75ml-24ID</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
+      <c r="D16" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="E16" s="5" t="n">
+        <v>763480</v>
+      </c>
       <c r="F16" s="5" t="n">
-        <v>763480</v>
+        <v>31812</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>31812</v>
+        <v>786384</v>
       </c>
       <c r="H16" s="5" t="n">
         <v>32766</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>40000</v>
       </c>
     </row>
     <row r="17">
@@ -27661,22 +27678,23 @@
           <t>Kiwi Shine Protect Neutral 30ml-48 ID</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="E17" s="5" t="n">
+        <v>761476</v>
+      </c>
       <c r="F17" s="5" t="n">
-        <v>761476</v>
+        <v>15864</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>15864</v>
+        <v>784320</v>
       </c>
       <c r="H17" s="5" t="n">
         <v>16340</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="18">
@@ -27693,22 +27711,23 @@
           <t>Kiwi Paste SP Brown 45ml-48ID</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n">
+      <c r="D18" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="E18" s="5" t="n">
+        <v>1001942</v>
+      </c>
       <c r="F18" s="5" t="n">
-        <v>1001942</v>
+        <v>20874</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>20874</v>
+        <v>1032000</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>21500</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>26300</v>
       </c>
     </row>
     <row r="19">
@@ -27725,22 +27744,23 @@
           <t>Kiwi Shine Protect Black 30ml-48 PH</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
+      <c r="D19" s="4" t="n">
         <v>48</v>
       </c>
+      <c r="E19" s="5" t="n">
+        <v>761476</v>
+      </c>
       <c r="F19" s="5" t="n">
-        <v>761476</v>
+        <v>15864</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>15864</v>
+        <v>784320</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>16340</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="20">
@@ -27757,22 +27777,23 @@
           <t>Kiwi Wax Rich SP Black 75ml-24ID</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n">
+      <c r="D20" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="E20" s="5" t="n">
+        <v>763480</v>
+      </c>
       <c r="F20" s="5" t="n">
-        <v>763480</v>
+        <v>31812</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>31812</v>
+        <v>786384</v>
       </c>
       <c r="H20" s="5" t="n">
         <v>32766</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>40000</v>
       </c>
     </row>
     <row r="21">
@@ -27789,22 +27810,23 @@
           <t>FrF Scm Choch Fsm Pou Jno 24x240g</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n">
+      <c r="D21" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="E21" s="5" t="n">
+        <v>181667</v>
+      </c>
       <c r="F21" s="5" t="n">
-        <v>181667</v>
+        <v>7569</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>7569</v>
+        <v>187117</v>
       </c>
       <c r="H21" s="5" t="n">
         <v>7797</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>9800</v>
       </c>
     </row>
     <row r="22">
@@ -27821,22 +27843,23 @@
           <t>FrF Scm Bkm Fsm Pou Jno 24x240g</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n">
+      <c r="D22" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="E22" s="5" t="n">
+        <v>181667</v>
+      </c>
       <c r="F22" s="5" t="n">
-        <v>181667</v>
+        <v>7569</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>7569</v>
+        <v>187117</v>
       </c>
       <c r="H22" s="5" t="n">
         <v>7797</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>9800</v>
       </c>
     </row>
     <row r="23">
@@ -27853,22 +27876,23 @@
           <t>BnB PWD BUBBLES 60G BTL-1310</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n">
+      <c r="D23" s="4" t="n">
         <v>36</v>
       </c>
+      <c r="E23" s="5" t="n">
+        <v>186120</v>
+      </c>
       <c r="F23" s="5" t="n">
-        <v>186120</v>
+        <v>5170</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>5170</v>
+        <v>191704</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>5325</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>6500</v>
       </c>
     </row>
     <row r="24">
@@ -27885,22 +27909,23 @@
           <t>Charm Cooling Fresh wing 23 cm 16 pads</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n">
+      <c r="D24" s="4" t="n">
         <v>24</v>
       </c>
+      <c r="E24" s="5" t="n">
+        <v>270524</v>
+      </c>
       <c r="F24" s="5" t="n">
-        <v>270524</v>
+        <v>11272</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>11272</v>
+        <v>278640</v>
       </c>
       <c r="H24" s="5" t="n">
         <v>11610</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>14200</v>
       </c>
     </row>
     <row r="25">
@@ -27917,22 +27942,23 @@
           <t>Mamy poko pants S1 kering pampers popok mamypoko</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n">
+      <c r="D25" s="4" t="n">
         <v>120</v>
       </c>
+      <c r="E25" s="5" t="n">
+        <v>107709</v>
+      </c>
       <c r="F25" s="5" t="n">
-        <v>107709</v>
+        <v>898</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>898</v>
+        <v>110940</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>924</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>13600</v>
       </c>
     </row>
     <row r="26">
@@ -27949,22 +27975,23 @@
           <t>MOLTO AIO BLUE (6+1) PROMO 216X18ML</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="n">
+      <c r="D26" s="4" t="n">
         <v>216</v>
       </c>
+      <c r="E26" s="5" t="n">
+        <v>155913</v>
+      </c>
       <c r="F26" s="5" t="n">
-        <v>155913</v>
+        <v>722</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>722</v>
+        <v>160590</v>
       </c>
       <c r="H26" s="5" t="n">
         <v>743</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>5500</v>
       </c>
     </row>
     <row r="27">
@@ -27981,22 +28008,23 @@
           <t>MOLTO AIO PINK (6+1) PROMO 216X18ML</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n">
+      <c r="D27" s="4" t="n">
         <v>216</v>
       </c>
+      <c r="E27" s="5" t="n">
+        <v>155913</v>
+      </c>
       <c r="F27" s="5" t="n">
-        <v>155913</v>
+        <v>722</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>722</v>
+        <v>160590</v>
       </c>
       <c r="H27" s="5" t="n">
         <v>743</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>5500</v>
       </c>
     </row>
     <row r="28">
@@ -28013,27 +28041,28 @@
           <t>RINSO ROYAL GOLD LIQUID 12+1 96X20G</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n">
+      <c r="D28" s="4" t="n">
         <v>96</v>
       </c>
+      <c r="E28" s="5" t="n">
+        <v>33758</v>
+      </c>
       <c r="F28" s="5" t="n">
-        <v>33758</v>
+        <v>352</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>352</v>
+        <v>34771</v>
       </c>
       <c r="H28" s="5" t="n">
         <v>362</v>
       </c>
+      <c r="I28" s="5" t="n">
+        <v>5400</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(scripts): fix rencengan modal calculation (x isi per renceng), use shopee product names for parsing
</commit_message>
<xml_diff>
--- a/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
+++ b/scripts/finance-reports/output/Laporan_Dana_Cair_Shopee_April_2026.xlsx
@@ -510,7 +510,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dibuat: 04/05/2026 15:01</t>
+          <t>Dibuat: 04/05/2026 15:13</t>
         </is>
       </c>
     </row>
@@ -24452,14 +24452,14 @@
         <v>5151</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>412</v>
+        <v>4944</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>4739</v>
+        <v>207</v>
       </c>
       <c r="Q6" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 4,739</t>
+          <t>DI ATAS TARGET +Rp 207</t>
         </is>
       </c>
     </row>
@@ -24517,14 +24517,14 @@
         <v>6089</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>412</v>
+        <v>4944</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>5677</v>
+        <v>1145</v>
       </c>
       <c r="Q9" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 5,677</t>
+          <t>DI ATAS TARGET +Rp 1,145</t>
         </is>
       </c>
     </row>
@@ -26935,14 +26935,14 @@
         <v>11626</v>
       </c>
       <c r="O83" s="5" t="n">
-        <v>924</v>
+        <v>9240</v>
       </c>
       <c r="P83" s="5" t="n">
-        <v>10702</v>
+        <v>2386</v>
       </c>
       <c r="Q83" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 10,702</t>
+          <t>DI ATAS TARGET +Rp 2,386</t>
         </is>
       </c>
     </row>
@@ -26998,144 +26998,144 @@
         <v>12251</v>
       </c>
       <c r="O84" s="5" t="n">
-        <v>924</v>
+        <v>9240</v>
       </c>
       <c r="P84" s="5" t="n">
-        <v>11327</v>
+        <v>3011</v>
       </c>
       <c r="Q84" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 11,327</t>
+          <t>DI ATAS TARGET +Rp 3,011</t>
         </is>
       </c>
     </row>
     <row r="85"/>
     <row r="86"/>
     <row r="87">
-      <c r="A87" s="4" t="n">
+      <c r="A87" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B87" s="12" t="inlineStr">
         <is>
           <t>UNMOL2709</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
+      <c r="C87" s="12" t="inlineStr">
         <is>
           <t>Molto Renceng 1000 Pelembut dan Pewangi Pakaian isi 6</t>
         </is>
       </c>
-      <c r="D87" s="4" t="inlineStr">
+      <c r="D87" s="12" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
+      <c r="E87" s="12" t="inlineStr">
         <is>
           <t>6+ pcs</t>
         </is>
       </c>
-      <c r="F87" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" s="4" t="n">
+      <c r="F87" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H87" s="5" t="n">
+      <c r="H87" s="13" t="n">
         <v>5450</v>
       </c>
-      <c r="I87" s="5" t="n">
+      <c r="I87" s="13" t="n">
         <v>491</v>
       </c>
-      <c r="J87" s="10" t="n">
+      <c r="J87" s="14" t="n">
         <v>9.009174311926605</v>
       </c>
-      <c r="K87" s="5" t="n">
+      <c r="K87" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="L87" s="10" t="n">
+      <c r="L87" s="14" t="n">
         <v>5.504587155963304</v>
       </c>
-      <c r="M87" s="5" t="n">
+      <c r="M87" s="13" t="n">
         <v>208</v>
       </c>
-      <c r="N87" s="5" t="n">
+      <c r="N87" s="13" t="n">
         <v>4451</v>
       </c>
-      <c r="O87" s="5" t="n">
-        <v>743</v>
-      </c>
-      <c r="P87" s="5" t="n">
-        <v>3708</v>
-      </c>
-      <c r="Q87" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 3,708</t>
+      <c r="O87" s="13" t="n">
+        <v>4458</v>
+      </c>
+      <c r="P87" s="13" t="n">
+        <v>-7</v>
+      </c>
+      <c r="Q87" s="12" t="inlineStr">
+        <is>
+          <t>DI BAWAH TARGET (RUGI Rp 7)</t>
         </is>
       </c>
     </row>
     <row r="88"/>
     <row r="89"/>
     <row r="90">
-      <c r="A90" s="4" t="n">
+      <c r="A90" s="12" t="n">
         <v>43</v>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="12" t="inlineStr">
         <is>
           <t>UNMOL2713</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="12" t="inlineStr">
         <is>
           <t>Molto Renceng 1000 Pelembut dan Pewangi Pakaian isi 6</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="D90" s="12" t="inlineStr">
         <is>
           <t>Pink</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E90" s="12" t="inlineStr">
         <is>
           <t>6+ pcs</t>
         </is>
       </c>
-      <c r="F90" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G90" s="4" t="n">
+      <c r="F90" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="H90" s="5" t="n">
+      <c r="H90" s="13" t="n">
         <v>5450</v>
       </c>
-      <c r="I90" s="5" t="n">
+      <c r="I90" s="13" t="n">
         <v>491</v>
       </c>
-      <c r="J90" s="10" t="n">
+      <c r="J90" s="14" t="n">
         <v>9.009174311926605</v>
       </c>
-      <c r="K90" s="5" t="n">
+      <c r="K90" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="L90" s="10" t="n">
+      <c r="L90" s="14" t="n">
         <v>5.504587155963304</v>
       </c>
-      <c r="M90" s="5" t="n">
+      <c r="M90" s="13" t="n">
         <v>208</v>
       </c>
-      <c r="N90" s="5" t="n">
+      <c r="N90" s="13" t="n">
         <v>4451</v>
       </c>
-      <c r="O90" s="5" t="n">
-        <v>743</v>
-      </c>
-      <c r="P90" s="5" t="n">
-        <v>3708</v>
-      </c>
-      <c r="Q90" s="11" t="inlineStr">
-        <is>
-          <t>DI ATAS TARGET +Rp 3,708</t>
+      <c r="O90" s="13" t="n">
+        <v>4458</v>
+      </c>
+      <c r="P90" s="13" t="n">
+        <v>-7</v>
+      </c>
+      <c r="Q90" s="12" t="inlineStr">
+        <is>
+          <t>DI BAWAH TARGET (RUGI Rp 7)</t>
         </is>
       </c>
     </row>
@@ -27193,14 +27193,14 @@
         <v>4377</v>
       </c>
       <c r="O93" s="5" t="n">
-        <v>362</v>
+        <v>4344</v>
       </c>
       <c r="P93" s="5" t="n">
-        <v>4015</v>
+        <v>33</v>
       </c>
       <c r="Q93" s="11" t="inlineStr">
         <is>
-          <t>DI ATAS TARGET +Rp 4,015</t>
+          <t>DI ATAS TARGET +Rp 33</t>
         </is>
       </c>
     </row>
@@ -27322,13 +27322,13 @@
         <v>460643</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>400</v>
+        <v>4798</v>
       </c>
       <c r="G6" s="5" t="n">
         <v>474462</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>412</v>
+        <v>4944</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>6100</v>
@@ -27355,13 +27355,13 @@
         <v>460643</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>400</v>
+        <v>4798</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>474462</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>412</v>
+        <v>4944</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>6100</v>
@@ -27949,13 +27949,13 @@
         <v>107709</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>898</v>
+        <v>8976</v>
       </c>
       <c r="G25" s="5" t="n">
         <v>110940</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>924</v>
+        <v>9240</v>
       </c>
       <c r="I25" s="5" t="n">
         <v>13600</v>
@@ -27982,13 +27982,13 @@
         <v>155913</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>722</v>
+        <v>4331</v>
       </c>
       <c r="G26" s="5" t="n">
         <v>160590</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>743</v>
+        <v>4458</v>
       </c>
       <c r="I26" s="5" t="n">
         <v>5500</v>
@@ -28015,13 +28015,13 @@
         <v>155913</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>722</v>
+        <v>4331</v>
       </c>
       <c r="G27" s="5" t="n">
         <v>160590</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>743</v>
+        <v>4458</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>5500</v>
@@ -28048,13 +28048,13 @@
         <v>33758</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>352</v>
+        <v>4220</v>
       </c>
       <c r="G28" s="5" t="n">
         <v>34771</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>362</v>
+        <v>4344</v>
       </c>
       <c r="I28" s="5" t="n">
         <v>5400</v>

</xml_diff>